<commit_message>
bdcom: Excel 重生成(cases 补 188,共 105)
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/bdcom/excel/bdcom_mirror_summary.xlsx
+++ b/data/bdcom/excel/bdcom_mirror_summary.xlsx
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -3043,7 +3043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D105"/>
+  <dimension ref="A1:D106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="2" max="2"/>
@@ -5011,17 +5011,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>597</t>
+          <t>188</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>BDCOM Powers Casablanca Port's Digital Transformation</t>
+          <t>Build smart transportation Boda scheme to help build a safe city in Ningde</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/597.html</t>
+          <t>https://bdcomnetworks.com/case/188.html</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -5033,17 +5033,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>597</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Yunnan Vocational College of Culture and Art (Woyunshan Campus)</t>
+          <t>BDCOM Powers Casablanca Port's Digital Transformation</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/85.html</t>
+          <t>https://bdcomnetworks.com/case/597.html</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -5055,17 +5055,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>85</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Progetto di infrastruttura wireless &amp; networking in ambiente Hospitality(Felix Olbia Hotel)</t>
+          <t>Yunnan Vocational College of Culture and Art (Woyunshan Campus)</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/86.html</t>
+          <t>https://bdcomnetworks.com/case/85.html</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -5077,17 +5077,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>86</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>BDCOM POL solution for Paraiso Residence Bukit Jalil</t>
+          <t>Progetto di infrastruttura wireless &amp; networking in ambiente Hospitality(Felix Olbia Hotel)</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/87.html</t>
+          <t>https://bdcomnetworks.com/case/86.html</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -5099,17 +5099,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Railway station Wi-Fi connection (Gujarat state)</t>
+          <t>BDCOM POL solution for Paraiso Residence Bukit Jalil</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/88.html</t>
+          <t>https://bdcomnetworks.com/case/87.html</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5121,17 +5121,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>88</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>FTTx Project in Kazan (Skynet)</t>
+          <t>Railway station Wi-Fi connection (Gujarat state)</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/89.html</t>
+          <t>https://bdcomnetworks.com/case/88.html</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5143,17 +5143,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>89</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Terminal Terrestre Daule Project</t>
+          <t>FTTx Project in Kazan (Skynet)</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/90.html</t>
+          <t>https://bdcomnetworks.com/case/89.html</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5165,17 +5165,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>91</t>
+          <t>90</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Implemented Intercity Ring Metro-E Network Backbone with BDCOM 100G Switches in Indonesia(PT TIS)</t>
+          <t>Terminal Terrestre Daule Project</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/91.html</t>
+          <t>https://bdcomnetworks.com/case/90.html</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -5187,17 +5187,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>91</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Wireless solution for CBD in Mohammedia city center</t>
+          <t>Implemented Intercity Ring Metro-E Network Backbone with BDCOM 100G Switches in Indonesia(PT TIS)</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/92.html</t>
+          <t>https://bdcomnetworks.com/case/91.html</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5209,17 +5209,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>93</t>
+          <t>92</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Punjab Prison Foundation Lahore Memo No/PPF/2021/302</t>
+          <t>Wireless solution for CBD in Mohammedia city center</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/93.html</t>
+          <t>https://bdcomnetworks.com/case/92.html</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5231,17 +5231,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>93</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Karbala TV core network reconstruction</t>
+          <t>Punjab Prison Foundation Lahore Memo No/PPF/2021/302</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/94.html</t>
+          <t>https://bdcomnetworks.com/case/93.html</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5253,17 +5253,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>94</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>FTTx Project in Cremia (Win Mobile)</t>
+          <t>Karbala TV core network reconstruction</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/95.html</t>
+          <t>https://bdcomnetworks.com/case/94.html</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5275,17 +5275,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>96</t>
+          <t>95</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Mzuzu university campus network</t>
+          <t>FTTx Project in Cremia (Win Mobile)</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/96.html</t>
+          <t>https://bdcomnetworks.com/case/95.html</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5297,17 +5297,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>96</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Vietnam-Cao Bang museum</t>
+          <t>Mzuzu university campus network</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/97.html</t>
+          <t>https://bdcomnetworks.com/case/96.html</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -5319,17 +5319,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>97</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Asia Mega Link FTTH</t>
+          <t>Vietnam-Cao Bang museum</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>https://bdcomnetworks.com/case/98.html</t>
+          <t>https://bdcomnetworks.com/case/97.html</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -5341,20 +5341,42 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
+          <t>98</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Asia Mega Link FTTH</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://bdcomnetworks.com/case/98.html</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
           <t>99</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B106" t="inlineStr">
         <is>
           <t>Baghdad Government Functional Building Network Upgrade</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t>https://bdcomnetworks.com/case/99.html</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
+      <c r="D106" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>

</xml_diff>